<commit_message>
Concept note: the occupancy table and the five-year table for all 25 settlements (blank after saturation, exact fill year); both as workbook sheets
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/W13/analysis/W13_growth_by_settlement.xlsx
+++ b/W13/analysis/W13_growth_by_settlement.xlsx
@@ -17,6 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook projection" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overflow routes" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Five-year to saturation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Five-year Qadf" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Occupancy" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1519,7 +1522,6 @@
       <c r="F19" t="n">
         <v>0</v>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>24</v>
       </c>
@@ -2056,6 +2058,2974 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2035</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2040</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2045</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>2060</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>2065</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>2075</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Saturation year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IBRI</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>67094</v>
+      </c>
+      <c r="C2" t="n">
+        <v>68702</v>
+      </c>
+      <c r="D2" t="n">
+        <v>78086</v>
+      </c>
+      <c r="E2" t="n">
+        <v>88257</v>
+      </c>
+      <c r="F2" t="n">
+        <v>100049</v>
+      </c>
+      <c r="G2" t="n">
+        <v>110330</v>
+      </c>
+      <c r="H2" t="n">
+        <v>122514</v>
+      </c>
+      <c r="I2" t="n">
+        <v>137057</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AD DARIZ</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11852</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12136</v>
+      </c>
+      <c r="D3" t="n">
+        <v>13794</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15590</v>
+      </c>
+      <c r="F3" t="n">
+        <v>17673</v>
+      </c>
+      <c r="G3" t="n">
+        <v>19490</v>
+      </c>
+      <c r="H3" t="n">
+        <v>21642</v>
+      </c>
+      <c r="I3" t="n">
+        <v>24211</v>
+      </c>
+      <c r="J3" t="n">
+        <v>27246</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AL ARAQI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10698</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10954</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12451</v>
+      </c>
+      <c r="E4" t="n">
+        <v>14072</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15953</v>
+      </c>
+      <c r="G4" t="n">
+        <v>17592</v>
+      </c>
+      <c r="H4" t="n">
+        <v>19535</v>
+      </c>
+      <c r="I4" t="n">
+        <v>21854</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="n">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AL AYNAYN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4553</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4662</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5299</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5989</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6789</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7487</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8314</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9301</v>
+      </c>
+      <c r="J5" t="n">
+        <v>12012</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AL WAHRAH</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3351</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3431</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3900</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4408</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4997</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5510</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6119</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6845</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7703</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8684</v>
+      </c>
+      <c r="L6" t="n">
+        <v>9803</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AT TAYYIB</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3349</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3429</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3898</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4405</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4994</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5507</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6115</v>
+      </c>
+      <c r="I7" t="n">
+        <v>6841</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8131</v>
+      </c>
+      <c r="K7" t="n">
+        <v>17539</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>2069</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AD DIBAYSHI</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2724</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2789</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3170</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3583</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4062</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4479</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4974</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5564</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6262</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>2063</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AL JIBAYYAH</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2684</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2749</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3128</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3538</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4014</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4429</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4921</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5508</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6201</v>
+      </c>
+      <c r="K9" t="n">
+        <v>6985</v>
+      </c>
+      <c r="L9" t="n">
+        <v>8694</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>2072</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BAT</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2558</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2619</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2977</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3365</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3814</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4206</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4671</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TANAM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2116</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2167</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2463</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2783</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3155</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3480</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3864</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4322</v>
+      </c>
+      <c r="J11" t="n">
+        <v>4864</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5961</v>
+      </c>
+      <c r="L11" t="n">
+        <v>8895</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SAYH AL MASARRAT</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1828</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1872</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2127</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2405</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2726</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3006</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3338</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3734</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4202</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4750</v>
+      </c>
+      <c r="L12" t="n">
+        <v>6229</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>2072</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SUWAYDA AL MA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1559</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1596</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1814</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2051</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2325</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2564</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2847</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3185</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3584</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4035</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4543</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HIJAR</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1408</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1442</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1639</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1852</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2315</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2571</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AL JAHLI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1376</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1409</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1601</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1810</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2052</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2263</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2513</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2811</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3163</v>
+      </c>
+      <c r="K15" t="n">
+        <v>8264</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>2065</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AL GHUBAYRAH</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>644</v>
+      </c>
+      <c r="C16" t="n">
+        <v>659</v>
+      </c>
+      <c r="D16" t="n">
+        <v>750</v>
+      </c>
+      <c r="E16" t="n">
+        <v>847</v>
+      </c>
+      <c r="F16" t="n">
+        <v>960</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1059</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1176</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1756</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2576</v>
+      </c>
+      <c r="K16" t="n">
+        <v>3502</v>
+      </c>
+      <c r="L16" t="n">
+        <v>4546</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AL QURAYN</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>588</v>
+      </c>
+      <c r="C17" t="n">
+        <v>602</v>
+      </c>
+      <c r="D17" t="n">
+        <v>684</v>
+      </c>
+      <c r="E17" t="n">
+        <v>773</v>
+      </c>
+      <c r="F17" t="n">
+        <v>877</v>
+      </c>
+      <c r="G17" t="n">
+        <v>967</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1074</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1201</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8376</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AL AKHEEDAR</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>480</v>
+      </c>
+      <c r="C18" t="n">
+        <v>492</v>
+      </c>
+      <c r="D18" t="n">
+        <v>559</v>
+      </c>
+      <c r="E18" t="n">
+        <v>631</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AL MAKHTIBYAH</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>364</v>
+      </c>
+      <c r="C19" t="n">
+        <v>373</v>
+      </c>
+      <c r="D19" t="n">
+        <v>424</v>
+      </c>
+      <c r="E19" t="n">
+        <v>479</v>
+      </c>
+      <c r="F19" t="n">
+        <v>543</v>
+      </c>
+      <c r="G19" t="n">
+        <v>599</v>
+      </c>
+      <c r="H19" t="n">
+        <v>665</v>
+      </c>
+      <c r="I19" t="n">
+        <v>744</v>
+      </c>
+      <c r="J19" t="n">
+        <v>837</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1140</v>
+      </c>
+      <c r="L19" t="n">
+        <v>5288</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AL QALI</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>224</v>
+      </c>
+      <c r="C20" t="n">
+        <v>229</v>
+      </c>
+      <c r="D20" t="n">
+        <v>261</v>
+      </c>
+      <c r="E20" t="n">
+        <v>295</v>
+      </c>
+      <c r="F20" t="n">
+        <v>366</v>
+      </c>
+      <c r="G20" t="n">
+        <v>474</v>
+      </c>
+      <c r="H20" t="n">
+        <v>602</v>
+      </c>
+      <c r="I20" t="n">
+        <v>851</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1415</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SATWAH</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>165</v>
+      </c>
+      <c r="C21" t="n">
+        <v>169</v>
+      </c>
+      <c r="D21" t="n">
+        <v>192</v>
+      </c>
+      <c r="E21" t="n">
+        <v>217</v>
+      </c>
+      <c r="F21" t="n">
+        <v>246</v>
+      </c>
+      <c r="G21" t="n">
+        <v>271</v>
+      </c>
+      <c r="H21" t="n">
+        <v>301</v>
+      </c>
+      <c r="I21" t="n">
+        <v>337</v>
+      </c>
+      <c r="J21" t="n">
+        <v>625</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SHALASHIL</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>152</v>
+      </c>
+      <c r="C22" t="n">
+        <v>156</v>
+      </c>
+      <c r="D22" t="n">
+        <v>177</v>
+      </c>
+      <c r="E22" t="n">
+        <v>200</v>
+      </c>
+      <c r="F22" t="n">
+        <v>227</v>
+      </c>
+      <c r="G22" t="n">
+        <v>250</v>
+      </c>
+      <c r="H22" t="n">
+        <v>278</v>
+      </c>
+      <c r="I22" t="n">
+        <v>311</v>
+      </c>
+      <c r="J22" t="n">
+        <v>7004</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>USAYBUQ</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>91</v>
+      </c>
+      <c r="C23" t="n">
+        <v>93</v>
+      </c>
+      <c r="D23" t="n">
+        <v>106</v>
+      </c>
+      <c r="E23" t="n">
+        <v>120</v>
+      </c>
+      <c r="F23" t="n">
+        <v>136</v>
+      </c>
+      <c r="G23" t="n">
+        <v>150</v>
+      </c>
+      <c r="H23" t="n">
+        <v>166</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>2054</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WADI AL MANKAS</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>49</v>
+      </c>
+      <c r="C24" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" t="n">
+        <v>57</v>
+      </c>
+      <c r="E24" t="n">
+        <v>64</v>
+      </c>
+      <c r="F24" t="n">
+        <v>73</v>
+      </c>
+      <c r="G24" t="n">
+        <v>81</v>
+      </c>
+      <c r="H24" t="n">
+        <v>89</v>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="n">
+        <v>113</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2903</v>
+      </c>
+      <c r="L24" t="n">
+        <v>8576</v>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ASH SHIAB</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>47</v>
+      </c>
+      <c r="C25" t="n">
+        <v>48</v>
+      </c>
+      <c r="D25" t="n">
+        <v>55</v>
+      </c>
+      <c r="E25" t="n">
+        <v>62</v>
+      </c>
+      <c r="F25" t="n">
+        <v>70</v>
+      </c>
+      <c r="G25" t="n">
+        <v>77</v>
+      </c>
+      <c r="H25" t="n">
+        <v>86</v>
+      </c>
+      <c r="I25" t="n">
+        <v>96</v>
+      </c>
+      <c r="J25" t="n">
+        <v>107</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MIAYRID</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>24</v>
+      </c>
+      <c r="C26" t="n">
+        <v>24</v>
+      </c>
+      <c r="D26" t="n">
+        <v>24</v>
+      </c>
+      <c r="E26" t="n">
+        <v>24</v>
+      </c>
+      <c r="F26" t="n">
+        <v>24</v>
+      </c>
+      <c r="G26" t="n">
+        <v>24</v>
+      </c>
+      <c r="H26" t="n">
+        <v>24</v>
+      </c>
+      <c r="I26" t="n">
+        <v>24</v>
+      </c>
+      <c r="J26" t="n">
+        <v>24</v>
+      </c>
+      <c r="K26" t="n">
+        <v>24</v>
+      </c>
+      <c r="L26" t="n">
+        <v>24</v>
+      </c>
+      <c r="M26" t="n">
+        <v>24</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>119978</v>
+      </c>
+      <c r="C27" t="n">
+        <v>122852</v>
+      </c>
+      <c r="D27" t="n">
+        <v>139636</v>
+      </c>
+      <c r="E27" t="n">
+        <v>157820</v>
+      </c>
+      <c r="F27" t="n">
+        <v>178909</v>
+      </c>
+      <c r="G27" t="n">
+        <v>197294</v>
+      </c>
+      <c r="H27" t="n">
+        <v>219083</v>
+      </c>
+      <c r="I27" t="n">
+        <v>245087</v>
+      </c>
+      <c r="J27" t="n">
+        <v>275803</v>
+      </c>
+      <c r="K27" t="n">
+        <v>310526</v>
+      </c>
+      <c r="L27" t="n">
+        <v>349622</v>
+      </c>
+      <c r="M27" t="n">
+        <v>367649</v>
+      </c>
+      <c r="N27" t="n">
+        <v>2073</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2035</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2040</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2045</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>2060</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>2065</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>2075</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Saturation year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IBRI</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>11492.4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>11767.7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>13375.1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>15117.2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>17136.9</v>
+      </c>
+      <c r="G2" t="n">
+        <v>18897.8</v>
+      </c>
+      <c r="H2" t="n">
+        <v>20984.8</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23475.8</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AD DARIZ</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2030</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2078.6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2362.6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2670.3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3027.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3338.1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3706.8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4146.8</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4666.7</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AL ARAQI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1832.3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1876.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2132.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2410.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2732.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3013.1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3345.9</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3743</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="n">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AL AYNAYN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>779.8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>798.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>907.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1025.8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1162.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1282.4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1424</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1593</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2057.4</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AL WAHRAH</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>573.9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>587.7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>668</v>
+      </c>
+      <c r="E6" t="n">
+        <v>755</v>
+      </c>
+      <c r="F6" t="n">
+        <v>855.9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>943.8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1048</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1172.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1319.4</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1487.4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1679</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AT TAYYIB</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>799.4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>813.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>893.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>980.4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1081.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1169.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1273.3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1397.6</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1618.5</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3229.9</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>2069</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AD DIBAYSHI</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>480.9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>492.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>557.4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>628.1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>710.1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>781.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>866.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>967.4</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1086.9</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>2063</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AL JIBAYYAH</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>459.7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>470.9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>535.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>606</v>
+      </c>
+      <c r="F9" t="n">
+        <v>687.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>758.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>842.9</v>
+      </c>
+      <c r="I9" t="n">
+        <v>943.4</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1062.2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1196.4</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1489.2</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>2072</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BAT</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>438.1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>448.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>509.8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>576.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>653.3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>720.4</v>
+      </c>
+      <c r="H10" t="n">
+        <v>800</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TANAM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>427.8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>478.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>533.4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>597.1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>652.7</v>
+      </c>
+      <c r="H11" t="n">
+        <v>718.5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>797</v>
+      </c>
+      <c r="J11" t="n">
+        <v>889.8</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1077.7</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1580.2</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SAYH AL MASARRAT</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>313.1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>320.6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>364.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>411.9</v>
+      </c>
+      <c r="F12" t="n">
+        <v>466.9</v>
+      </c>
+      <c r="G12" t="n">
+        <v>514.9</v>
+      </c>
+      <c r="H12" t="n">
+        <v>571.7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>639.6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>719.8</v>
+      </c>
+      <c r="K12" t="n">
+        <v>813.6</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1066.9</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>2072</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SUWAYDA AL MA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>267</v>
+      </c>
+      <c r="C13" t="n">
+        <v>273.4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>310.8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>351.2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>398.2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>439.1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>487.6</v>
+      </c>
+      <c r="I13" t="n">
+        <v>545.5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>613.8</v>
+      </c>
+      <c r="K13" t="n">
+        <v>691.1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>778.1</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HIJAR</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>241.2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>246.9</v>
+      </c>
+      <c r="D14" t="n">
+        <v>280.7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>317.2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>359.6</v>
+      </c>
+      <c r="G14" t="n">
+        <v>396.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>440.4</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AL JAHLI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>235.7</v>
+      </c>
+      <c r="C15" t="n">
+        <v>241.3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>274.3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>310</v>
+      </c>
+      <c r="F15" t="n">
+        <v>351.4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>387.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>430.4</v>
+      </c>
+      <c r="I15" t="n">
+        <v>481.4</v>
+      </c>
+      <c r="J15" t="n">
+        <v>541.8</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1415.5</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>2065</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AL GHUBAYRAH</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>112.9</v>
+      </c>
+      <c r="D16" t="n">
+        <v>128.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>145.1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>164.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>181.4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>201.4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>300.8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>441.2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>599.9</v>
+      </c>
+      <c r="L16" t="n">
+        <v>778.6</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AL QURAYN</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>100.7</v>
+      </c>
+      <c r="C17" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>117.2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>150.2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>165.6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>183.9</v>
+      </c>
+      <c r="I17" t="n">
+        <v>205.7</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1434.7</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AL AKHEEDAR</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="C18" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="E18" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AL MAKHTIBYAH</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="C19" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="D19" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="E19" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>112.3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>121.8</v>
+      </c>
+      <c r="H19" t="n">
+        <v>133.1</v>
+      </c>
+      <c r="I19" t="n">
+        <v>146.7</v>
+      </c>
+      <c r="J19" t="n">
+        <v>162.6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>214.6</v>
+      </c>
+      <c r="L19" t="n">
+        <v>925</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AL QALI</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="C20" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="G20" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="H20" t="n">
+        <v>103</v>
+      </c>
+      <c r="I20" t="n">
+        <v>145.8</v>
+      </c>
+      <c r="J20" t="n">
+        <v>242.4</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SATWAH</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>29</v>
+      </c>
+      <c r="D21" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="E21" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="I21" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="J21" t="n">
+        <v>107</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SHALASHIL</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>26</v>
+      </c>
+      <c r="C22" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D22" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="G22" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="H22" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="I22" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1199.7</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>USAYBUQ</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="C23" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D23" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="G23" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="H23" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>2054</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WADI AL MANKAS</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C24" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E24" t="n">
+        <v>11</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="H24" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="I24" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>497.2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1468.9</v>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ASH SHIAB</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D25" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="F25" t="n">
+        <v>12</v>
+      </c>
+      <c r="G25" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H25" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="I25" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="J25" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MIAYRID</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M26" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>20866</v>
+      </c>
+      <c r="C27" t="n">
+        <v>21359</v>
+      </c>
+      <c r="D27" t="n">
+        <v>24233</v>
+      </c>
+      <c r="E27" t="n">
+        <v>27348</v>
+      </c>
+      <c r="F27" t="n">
+        <v>30960</v>
+      </c>
+      <c r="G27" t="n">
+        <v>34109</v>
+      </c>
+      <c r="H27" t="n">
+        <v>37841</v>
+      </c>
+      <c r="I27" t="n">
+        <v>42295</v>
+      </c>
+      <c r="J27" t="n">
+        <v>47556</v>
+      </c>
+      <c r="K27" t="n">
+        <v>53504</v>
+      </c>
+      <c r="L27" t="n">
+        <v>60200</v>
+      </c>
+      <c r="M27" t="n">
+        <v>63288</v>
+      </c>
+      <c r="N27" t="n">
+        <v>2073</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SETTLE</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>properties</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>workbook_2024</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>OR_raw</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>OR_used</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>people_used</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>delta_vs_workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IBRI</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>11052</v>
+      </c>
+      <c r="C2" t="n">
+        <v>67105.50878491651</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="F2" t="n">
+        <v>58663</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-8443</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AD DARIZ</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2439</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11849.67146371732</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12937</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1087</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AL ARAQI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2466</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10695.67732032832</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="F4" t="n">
+        <v>13087</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AL AYNAYN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>889</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4554.030567590516</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4716</v>
+      </c>
+      <c r="G5" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AL WAHRAH</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>716</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3351.079096906229</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3799</v>
+      </c>
+      <c r="G6" t="n">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AT TAYYIB</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>833</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3348.081709520803</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4418</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AL JIBAYYAH</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>524</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2685.659097341665</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G8" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BAT</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>418</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2556.771439768348</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2218</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-339</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AD DIBAYSHI</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>681</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2410.898587010952</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3613</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1202</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TANAM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>403</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2116.155494110731</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2140</v>
+      </c>
+      <c r="G11" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SUWAYDA AL MA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>301</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1558.641440421502</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1598</v>
+      </c>
+      <c r="G12" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HIJAR</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>352</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1033.099518843483</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1868</v>
+      </c>
+      <c r="G13" t="n">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AL GHUBAYRAH</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>161</v>
+      </c>
+      <c r="C14" t="n">
+        <v>631.4496091964032</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>854</v>
+      </c>
+      <c r="G14" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AL QURAYN</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>147</v>
+      </c>
+      <c r="C15" t="n">
+        <v>548.5218915329516</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>779</v>
+      </c>
+      <c r="G15" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SAYH AL MASARRAT</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>457</v>
+      </c>
+      <c r="C16" t="n">
+        <v>465.5941738694999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2429</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1963</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AL JAHLI</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>344</v>
+      </c>
+      <c r="C17" t="n">
+        <v>414.6385883172585</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1828</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1413</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SATWAH</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>27</v>
+      </c>
+      <c r="C18" t="n">
+        <v>262.7709607890096</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="E18" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="F18" t="n">
+        <v>143</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AL AKHEEDAR</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>120</v>
+      </c>
+      <c r="C19" t="n">
+        <v>197.8275674381137</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" t="n">
+        <v>638</v>
+      </c>
+      <c r="G19" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AL QALI</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>56</v>
+      </c>
+      <c r="C20" t="n">
+        <v>190.8336635387865</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>297</v>
+      </c>
+      <c r="G20" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SHALASHIL</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>38</v>
+      </c>
+      <c r="C21" t="n">
+        <v>129.8867867017918</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>202</v>
+      </c>
+      <c r="G21" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AL MAKHTIBYAH</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>91</v>
+      </c>
+      <c r="C22" t="n">
+        <v>121.8937536739892</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" t="n">
+        <v>483</v>
+      </c>
+      <c r="G22" t="n">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>USAYBUQ</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" t="n">
+        <v>90.92075069125428</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="F23" t="n">
+        <v>111</v>
+      </c>
+      <c r="G23" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WADI AL MANKAS</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>51.95471468071673</v>
+      </c>
+      <c r="D24" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="F24" t="n">
+        <v>42</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ASH SHIAB</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>11</v>
+      </c>
+      <c r="C25" t="n">
+        <v>46.95906903834011</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="F25" t="n">
+        <v>58</v>
+      </c>
+      <c r="G25" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MIAYRID</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n">
+        <v>33.97039036816093</v>
+      </c>
+      <c r="D26" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="E26" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="F26" t="n">
+        <v>21</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>